<commit_message>
fix(lab1): normalize ISO25010 NFR categories
</commit_message>
<xml_diff>
--- a/docs/lab1/source/计算机23-2_231002208_戚晋瑜_实验一_GlossaryRTM_v1.0.xlsx
+++ b/docs/lab1/source/计算机23-2_231002208_戚晋瑜_实验一_GlossaryRTM_v1.0.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="1" r:id="R914a364b2b334983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="Rcadc275259a44b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naming" sheetId="3" r:id="Ra320588ee4d74a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="1" r:id="Rbf60a163dd1542df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="2" r:id="R5501fed091d34d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Naming" sheetId="3" r:id="R523bb07ec712462a"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>